<commit_message>
Add LinkedIn post for top leadership consultants for nonprofits
</commit_message>
<xml_diff>
--- a/blog-data/linkedin-posts-tracker.xlsx
+++ b/blog-data/linkedin-posts-tracker.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -488,6 +488,42 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>17 Top Leadership Consultants for Nonprofits (2026)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/17-top-leadership-consultants-for-nonprofits-2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>blog-images/blog-top-leadership-consultants-nonprofits-20260324/linkedin-post.md</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>37</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Commercial listicle. 37 tags across 4 tiers.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update LinkedIn posts tracker
</commit_message>
<xml_diff>
--- a/blog-data/linkedin-posts-tracker.xlsx
+++ b/blog-data/linkedin-posts-tracker.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -509,7 +509,6 @@
           <t>2026-03-24</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>READY</t>
@@ -521,6 +520,42 @@
       <c r="H2" t="inlineStr">
         <is>
           <t>Commercial listicle. 37 tags across 4 tiers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>50 Best Keynote Speakers for Church Leaders (2026)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/50-best-keynote-speakers-for-church-leaders-2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>blog-images/blog-best-keynote-speakers-church-leaders-20260324/linkedin-post.md</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>45</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>45 people tagged from blog list</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update LinkedIn tracker for aged care speakers post
</commit_message>
<xml_diff>
--- a/blog-data/linkedin-posts-tracker.xlsx
+++ b/blog-data/linkedin-posts-tracker.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -544,7 +544,6 @@
           <t>2026-03-24</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>READY</t>
@@ -558,6 +557,38 @@
           <t>45 people tagged from blog list</t>
         </is>
       </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>50 Best Leadership Speakers for Aged Care (2026)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/50-best-leadership-speakers-for-aged-care-2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>blog-images/blog-best-leadership-speakers-aged-care-20260324/linkedin-post.md</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>45</v>
+      </c>
+      <c r="H4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add LinkedIn post for best leadership speakers for hospitals
</commit_message>
<xml_diff>
--- a/blog-data/linkedin-posts-tracker.xlsx
+++ b/blog-data/linkedin-posts-tracker.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -522,6 +522,38 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>50 Best Leadership Speakers for Hospitals (2026)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/50-best-leadership-speakers-for-hospitals-2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>blog-images/blog-best-leadership-speakers-hospitals-20260324/linkedin-post.md</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>47</v>
+      </c>
+      <c r="H3" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add LinkedIn post for top leadership consultants for healthcare
</commit_message>
<xml_diff>
--- a/blog-data/linkedin-posts-tracker.xlsx
+++ b/blog-data/linkedin-posts-tracker.xlsx
@@ -560,12 +560,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.consultclarity.org/post/50-top-leadership-consultants-for-healthcare-2026-1</t>
+          <t>https://www.consultclarity.org/post/50-top-leadership-consultants-for-healthcare-2026</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>linkedin-post-50-top-leadership-consultants-for-healthcare-2026.md</t>
+          <t>blog-images/blog-top-leadership-consultants-healthcare-20260325/linkedin-post.md</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -580,11 +580,11 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>41</v>
+        <v>18</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>COMMERCIAL listicle. 22 featured people + 19 additional thought leaders tagged.</t>
+          <t>Commercial listicle, adjacent fit</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add LinkedIn post for top leadership consultants for construction
</commit_message>
<xml_diff>
--- a/blog-data/linkedin-posts-tracker.xlsx
+++ b/blog-data/linkedin-posts-tracker.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -608,7 +608,6 @@
           <t>2026-03-25</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>READY</t>
@@ -622,6 +621,38 @@
           <t>COMMERCIAL listicle, ADJACENT fit</t>
         </is>
       </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>50 Top Leadership Consultants for Construction (2026)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/50-top-leadership-consultants-for-construction-2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>linkedin-post-top-leadership-consultants-for-construction.md</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>22</v>
+      </c>
+      <c r="H6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add LinkedIn post for best leadership speakers mining companies
</commit_message>
<xml_diff>
--- a/blog-data/linkedin-posts-tracker.xlsx
+++ b/blog-data/linkedin-posts-tracker.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -643,7 +643,6 @@
           <t>2026-03-25</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>READY</t>
@@ -652,7 +651,42 @@
       <c r="G6" t="n">
         <v>22</v>
       </c>
-      <c r="H6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>50 Best Leadership Speakers for Mining Companies (2026)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/50-best-leadership-speakers-for-mining-companies-2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>blog-images/blog-best-leadership-speakers-mining-companies-20260325/linkedin-post.md</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>37</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Commercial listicle, mining leadership speakers</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add LinkedIn post for top leadership consultants for mining
</commit_message>
<xml_diff>
--- a/blog-data/linkedin-posts-tracker.xlsx
+++ b/blog-data/linkedin-posts-tracker.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -673,7 +673,6 @@
           <t>2026-03-25</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>READY</t>
@@ -685,6 +684,42 @@
       <c r="H7" t="inlineStr">
         <is>
           <t>Commercial listicle, mining leadership speakers</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>50 Top Leadership Consultants for Mining (2026)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/50-top-leadership-consultants-for-mining-2026</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>linkedin-post-top-leadership-consultants-for-mining.md</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>45</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>50 consultants. Full content published to Wix.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add LinkedIn post for best leadership speakers agriculture
</commit_message>
<xml_diff>
--- a/blog-data/linkedin-posts-tracker.xlsx
+++ b/blog-data/linkedin-posts-tracker.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -708,7 +708,6 @@
           <t>2026-03-25</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>READY</t>
@@ -722,6 +721,38 @@
           <t>50 consultants. Full content published to Wix.</t>
         </is>
       </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>50 Best Leadership Speakers for Agriculture (2026)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/50-best-leadership-speakers-for-agriculture-2026</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>linkedin-post-best-leadership-speakers-agriculture.md</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>37</v>
+      </c>
+      <c r="H9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add LinkedIn post for agribusiness blog
</commit_message>
<xml_diff>
--- a/blog-data/linkedin-posts-tracker.xlsx
+++ b/blog-data/linkedin-posts-tracker.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -743,7 +743,6 @@
           <t>2026-03-25</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>READY</t>
@@ -752,7 +751,38 @@
       <c r="G9" t="n">
         <v>37</v>
       </c>
-      <c r="H9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>50 Top Leadership Consultants for Agribusiness (2026)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/50-top-leadership-consultants-for-agribusiness-2026</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>linkedin-post-top-leadership-consultants-agribusiness.md</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>22</v>
+      </c>
+      <c r="H10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add LinkedIn post for hospitality thought leaders
</commit_message>
<xml_diff>
--- a/blog-data/linkedin-posts-tracker.xlsx
+++ b/blog-data/linkedin-posts-tracker.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -803,7 +803,6 @@
           <t>2026-03-25</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>READY</t>
@@ -812,7 +811,42 @@
       <c r="G11" t="n">
         <v>49</v>
       </c>
-      <c r="H11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>50 Best Thought Leaders in Hospitality (2026)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/50-best-thought-leaders-in-hospitality-2026</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>blog-images/blog-thought-leaders-hospitality-20260325/linkedin-post.md</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>44</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Commercial, Adjacent fit</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add LinkedIn post for thought leaders in engineering
</commit_message>
<xml_diff>
--- a/blog-data/linkedin-posts-tracker.xlsx
+++ b/blog-data/linkedin-posts-tracker.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -833,7 +833,6 @@
           <t>2026-03-25</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>READY</t>
@@ -847,6 +846,38 @@
           <t>Commercial, Adjacent fit</t>
         </is>
       </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>50 Best Thought Leaders in Engineering (2026)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/50-best-thought-leaders-in-engineering-2026</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>blog-images/blog-thought-leaders-engineering-20260325/linkedin-post.md</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>48</v>
+      </c>
+      <c r="H13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add LinkedIn post for thought leaders in architecture
</commit_message>
<xml_diff>
--- a/blog-data/linkedin-posts-tracker.xlsx
+++ b/blog-data/linkedin-posts-tracker.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -868,7 +868,6 @@
           <t>2026-03-25</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>READY</t>
@@ -877,7 +876,42 @@
       <c r="G13" t="n">
         <v>48</v>
       </c>
-      <c r="H13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>50 Best Thought Leaders in Architecture (2026)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/50-best-thought-leaders-in-architecture-2026</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>linkedin-post-best-thought-leaders-in-architecture.md</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>44</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>COMMERCIAL listicle, architecture thought leaders</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add LinkedIn post for best thought leaders in retail
</commit_message>
<xml_diff>
--- a/blog-data/linkedin-posts-tracker.xlsx
+++ b/blog-data/linkedin-posts-tracker.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -898,7 +898,6 @@
           <t>2026-03-26</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>READY</t>
@@ -910,6 +909,42 @@
       <c r="H14" t="inlineStr">
         <is>
           <t>COMMERCIAL listicle, architecture thought leaders</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>50 Best Thought Leaders in Retail (2026)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/50-best-thought-leaders-in-retail-2026</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>linkedin-post-best-thought-leaders-in-retail.md</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>47</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Full pipeline</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add LinkedIn post for thought leaders in real estate
</commit_message>
<xml_diff>
--- a/blog-data/linkedin-posts-tracker.xlsx
+++ b/blog-data/linkedin-posts-tracker.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -933,7 +933,6 @@
           <t>2026-03-26</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>READY</t>
@@ -947,6 +946,38 @@
           <t>Full pipeline</t>
         </is>
       </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>50 Best Thought Leaders in Real Estate (2026)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/50-best-thought-leaders-in-real-estate-2026</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>linkedin-post-50-best-thought-leaders-in-real-estate-2026.md</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>48</v>
+      </c>
+      <c r="H16" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update LinkedIn tracker for manufacturing thought leaders
</commit_message>
<xml_diff>
--- a/blog-data/linkedin-posts-tracker.xlsx
+++ b/blog-data/linkedin-posts-tracker.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -968,7 +968,6 @@
           <t>2026-03-26</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>READY</t>
@@ -977,7 +976,42 @@
       <c r="G16" t="n">
         <v>48</v>
       </c>
-      <c r="H16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>50 Best Thought Leaders in Manufacturing (2026)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/50-best-thought-leaders-in-manufacturing-2026</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>blog-images/blog-thought-leaders-manufacturing-20260326/linkedin-post.md</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>48</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>48 people tagged. Full pipeline complete.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update LinkedIn tracker: agriculture thought leaders
</commit_message>
<xml_diff>
--- a/blog-data/linkedin-posts-tracker.xlsx
+++ b/blog-data/linkedin-posts-tracker.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -998,7 +998,6 @@
           <t>2026-03-26</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>READY</t>
@@ -1012,6 +1011,38 @@
           <t>48 people tagged. Full pipeline complete.</t>
         </is>
       </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>50 Best Thought Leaders in Agriculture (2026)</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/50-best-thought-leaders-in-agriculture-2026</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>blog-images/blog-thought-leaders-agriculture-20260326/linkedin-post.md</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>42</v>
+      </c>
+      <c r="H18" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update LinkedIn tracker: thought leaders in mining
</commit_message>
<xml_diff>
--- a/blog-data/linkedin-posts-tracker.xlsx
+++ b/blog-data/linkedin-posts-tracker.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1033,7 +1033,6 @@
           <t>2026-03-26</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
           <t>READY</t>
@@ -1042,7 +1041,38 @@
       <c r="G18" t="n">
         <v>42</v>
       </c>
-      <c r="H18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>50 Best Thought Leaders in Mining (2026)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/50-best-thought-leaders-in-mining-2026</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>blog-images/blog-thought-leaders-mining-20260326/linkedin-post.md</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>46</v>
+      </c>
+      <c r="H19" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add LinkedIn post for best thought leaders in healthcare
</commit_message>
<xml_diff>
--- a/blog-data/linkedin-posts-tracker.xlsx
+++ b/blog-data/linkedin-posts-tracker.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1063,7 +1063,6 @@
           <t>2026-03-26</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
           <t>READY</t>
@@ -1072,7 +1071,42 @@
       <c r="G19" t="n">
         <v>46</v>
       </c>
-      <c r="H19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>50 Best Thought Leaders in Healthcare (2026)</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/50-best-thought-leaders-in-healthcare-2026</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>linkedin-post-best-thought-leaders-in-healthcare.md</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>48</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Commercial listicle, all 50 featured people tagged</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add LinkedIn post for insurance thought leaders
</commit_message>
<xml_diff>
--- a/blog-data/linkedin-posts-tracker.xlsx
+++ b/blog-data/linkedin-posts-tracker.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1093,7 +1093,6 @@
           <t>2026-03-26</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
           <t>READY</t>
@@ -1107,6 +1106,38 @@
           <t>Commercial listicle, all 50 featured people tagged</t>
         </is>
       </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>50 Best Thought Leaders in Insurance (2026)</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/50-best-thought-leaders-in-insurance-2026</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>linkedin-post-best-thought-leaders-in-insurance.md</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>49</v>
+      </c>
+      <c r="H21" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add LinkedIn post for thought leaders in consulting
</commit_message>
<xml_diff>
--- a/blog-data/linkedin-posts-tracker.xlsx
+++ b/blog-data/linkedin-posts-tracker.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1128,7 +1128,6 @@
           <t>2026-03-26</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
           <t>READY</t>
@@ -1137,7 +1136,42 @@
       <c r="G21" t="n">
         <v>49</v>
       </c>
-      <c r="H21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>50 Best Thought Leaders in Consulting (2026)</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/50-best-thought-leaders-in-consulting-2026</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>blog-images/blog-thought-leaders-consulting-20260326/linkedin-post.md</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>41</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>41 tags in post</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add blog images and LinkedIn tracker for technology thought leaders
</commit_message>
<xml_diff>
--- a/blog-data/linkedin-posts-tracker.xlsx
+++ b/blog-data/linkedin-posts-tracker.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1158,7 +1158,6 @@
           <t>2026-03-26</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
           <t>READY</t>
@@ -1170,6 +1169,42 @@
       <c r="H22" t="inlineStr">
         <is>
           <t>41 tags in post</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>50 Best Thought Leaders in Technology (2026)</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/50-best-thought-leaders-in-technology-2026</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>linkedin-post-best-thought-leaders-in-technology.md</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>49</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>All 49 featured people tagged (excluding Jonno)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add LinkedIn post for best thought leaders in artificial intelligence
</commit_message>
<xml_diff>
--- a/blog-data/linkedin-posts-tracker.xlsx
+++ b/blog-data/linkedin-posts-tracker.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1193,7 +1193,6 @@
           <t>2026-03-26</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
           <t>READY</t>
@@ -1205,6 +1204,42 @@
       <c r="H23" t="inlineStr">
         <is>
           <t>All 49 featured people tagged (excluding Jonno)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>50 Best Thought Leaders in Artificial Intelligence (2026)</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/50-best-thought-leaders-in-artificial-intelligence-2026</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>blog-images/blog-best-thought-leaders-in-artificial-intelligence-20260327/linkedin-post.md</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>49</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>All 49 featured people tagged</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add LinkedIn post for software engineering thought leaders
</commit_message>
<xml_diff>
--- a/blog-data/linkedin-posts-tracker.xlsx
+++ b/blog-data/linkedin-posts-tracker.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1228,7 +1228,6 @@
           <t>2026-03-27</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
           <t>READY</t>
@@ -1242,6 +1241,38 @@
           <t>All 49 featured people tagged</t>
         </is>
       </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>50 Best Thought Leaders in Software Engineering (2026)</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/50-best-thought-leaders-in-software-engineering-2026</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>linkedin-post.md</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>49</v>
+      </c>
+      <c r="H25" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add LinkedIn post for best thought leaders in product management
</commit_message>
<xml_diff>
--- a/blog-data/linkedin-posts-tracker.xlsx
+++ b/blog-data/linkedin-posts-tracker.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1263,7 +1263,6 @@
           <t>2026-03-27</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
           <t>READY</t>
@@ -1272,7 +1271,42 @@
       <c r="G25" t="n">
         <v>49</v>
       </c>
-      <c r="H25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>50 Best Thought Leaders in Product Management (2026)</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/50-best-thought-leaders-in-product-management-2026</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>linkedin-post-best-thought-leaders-in-product-management.md</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>49</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>49 people tagged in the LinkedIn post</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>